<commit_message>
feat(combat): expand Reach sliders up to 10.0 blocks for combat and 12.0 blocks for block placement
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Progetti AI\Aetheris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D90A69D-660D-4C2E-808C-287B2A9A9892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C36C91-3C02-4350-8A00-F9188E87C50A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11730" yWindow="195" windowWidth="16425" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14340" yWindow="90" windowWidth="16425" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aetheris Checklist" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="77">
   <si>
     <t>Categoria</t>
   </si>
@@ -696,7 +696,9 @@
       <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -709,7 +711,9 @@
       <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix(reach): bypass wall raycast obstacle and expand KillAura range to 15.0 blocks for TP-Reach
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Progetti AI\Aetheris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C36C91-3C02-4350-8A00-F9188E87C50A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6112B53E-0E1A-484E-A9B4-90E7DEA7DC4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14340" yWindow="90" windowWidth="16425" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="78">
   <si>
     <t>Categoria</t>
   </si>
@@ -256,6 +256,9 @@
   </si>
   <si>
     <t>SI</t>
+  </si>
+  <si>
+    <t>NO</t>
   </si>
 </sst>
 </file>
@@ -712,7 +715,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E5" s="3"/>
     </row>

</xml_diff>

<commit_message>
fix(reach): re-add custom raycast to bypass vanilla block interaction caps
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Progetti AI\Aetheris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479E2DCC-007F-43E2-9E0A-D730AD124203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA9A6D4-9B46-4714-9A8B-3AAADF37CEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14340" yWindow="90" windowWidth="16425" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7590" yWindow="60" windowWidth="16425" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aetheris Checklist" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
fix(surround,nofall): fix NoFall packet spoofing and overhaul Surround module with player centering and neighbor detection
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Progetti AI\Aetheris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA9A6D4-9B46-4714-9A8B-3AAADF37CEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A31011E-8E13-4813-93B2-2FA73175F61C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7590" yWindow="60" windowWidth="16425" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12330" yWindow="165" windowWidth="16425" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aetheris Checklist" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="79">
   <si>
     <t>Categoria</t>
   </si>
@@ -259,6 +259,9 @@
   </si>
   <si>
     <t>NO</t>
+  </si>
+  <si>
+    <t>a volte si a volte no</t>
   </si>
 </sst>
 </file>
@@ -715,7 +718,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E5" s="3"/>
     </row>
@@ -729,7 +732,9 @@
       <c r="C6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -742,7 +747,9 @@
       <c r="C7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -755,7 +762,9 @@
       <c r="C8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="2"/>
+      <c r="D8" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -768,8 +777,12 @@
       <c r="C9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="3"/>
+      <c r="D9" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -781,7 +794,9 @@
       <c r="C10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="2"/>
+      <c r="D10" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -794,7 +809,9 @@
       <c r="C11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -807,7 +824,9 @@
       <c r="C12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="2"/>
+      <c r="D12" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="E12" s="3"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -820,7 +839,9 @@
       <c r="C13" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="2"/>
+      <c r="D13" s="2" t="s">
+        <v>77</v>
+      </c>
       <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Implement Roadmap Batch: CameraClip, Trajectories, AirPlace, InventorySort, BedTrap, CrystalAura auto-placement, StorageESP hideEmpty, and update docs
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1515,110 +1515,245 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Movement</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>BunnyJump</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Salta automaticamente all'atterraggio durante il movimento</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>Batch 2026-08</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Movement</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Jetpack</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Vola verso l'alto tenendo premuto Spazio con effetto fiamme</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Batch 2026-08</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Movement</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Sneak</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Mantiene il giocatore accovacciato in modo permanente</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Batch 2026-08</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>AutoFarm</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Raccoglie le colture mature e le risemina automaticamente</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Batch 2026-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Render</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>CameraClip</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Impedisce alla telecamera in terza persona di clippare nei blocchi</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Batch 2026-08 (Roadmap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Render</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Trajectories</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Disegna in 3D la traiettoria parabolica di frecce, perle e proiettili</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Batch 2026-08 (Roadmap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>AirPlace</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Permette di piazzare blocchi a sbalzo nel vuoto senza blocco di supporto</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Batch 2026-08 (Roadmap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>InventorySort</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Ordina automaticamente gli oggetti nell'inventario e nei contenitori</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Batch 2026-08 (Roadmap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Combat</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>BedTrap</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Piazza ed esplode automaticamente i letti nel Nether/End per PvP</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Batch 2026-08 (Roadmap)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement 9 new modules from Qwen3.8-max conceptual mapping, update Excel checklist and docs to 61 total modules
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1757,6 +1757,249 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>AutoBrewer</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Gestisce automaticamente l'inserimento di ingredienti e fiamme negli alambicchi</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Mappatura Qwen3.8-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AutoSmelter</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Automatizza l'inserimento di prodotti e carburante nei forni</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Mappatura Qwen3.8-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>StrongholdFinder</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Calcola le coordinate X, Z della fortezza triangolando 2 Occhi di Ender</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Mappatura Qwen3.8-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PacketLogger</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Registra i pacchetti di rete C2S e S2C inviati/ricevuti per debug</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Mappatura Qwen3.8-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>ServerFinder</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Scansiona IP in background alla ricerca di server Minecraft attivi</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Mappatura Qwen3.8-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Render</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Waypoints</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Consente di impostare e visualizzare marcatori 3D con fasci di luce beacon</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Mappatura Qwen3.8-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>NoChatReports</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Disabilita le firme digitali sui messaggi inviati in chat per la privacy</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Mappatura Qwen3.8-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Combat</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>BowAimbot</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Mantiene la mira automatica con l'arco calcolando parabola e anticipo</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Mappatura Qwen3.8-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>AutoWalk</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Mantiene la camminata in avanti automatica</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Mappatura Qwen3.8-max</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Integrate and verify Qwen2.5 changes: PluginScanner, ChatSignatureMixin, ConnectionMixin performance caching, and doc updates
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2000,6 +2000,33 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>PluginScanner</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Scansiona /plugins e comandi del server per identificare PEX, LuckPerms, etc.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Aggiunto da Qwen2.5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Update Excel checklist with AntiDetect and sync AGENTS.md total modules to 62
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2027,6 +2027,33 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>AntiDetect</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Spoofa il brand del client in vanilla e rimuove i payload fabric:*</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Integrato</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
docs: sync AGENTS/CLAUDE with audit tool, hot-path pattern, module list
Adds tools/aetheris_server_audit.py to key files, documents O(1) module index rule for mixins, Player list now 12 (PermissionViewer), checklist row added.
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11955" yWindow="945" windowWidth="16425" windowHeight="13875" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aetheris Checklist" sheetId="1" state="visible" r:id="rId1"/>
@@ -72,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -82,6 +82,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,13 +454,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" style="4" min="1" max="1"/>
+    <col width="20" customWidth="1" style="4" min="2" max="2"/>
     <col width="63.85546875" customWidth="1" style="3" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" style="4" min="4" max="4"/>
     <col width="40" customWidth="1" style="3" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1623,434 +1629,488 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Render</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>CameraClip</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Impedisce alla telecamera in terza persona di clippare nei blocchi</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>Batch 2026-08 (Roadmap)</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>Render</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>Trajectories</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>Disegna in 3D la traiettoria parabolica di frecce, perle e proiettili</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>Batch 2026-08 (Roadmap)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>AirPlace</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>Permette di piazzare blocchi a sbalzo nel vuoto senza blocco di supporto</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>Batch 2026-08 (Roadmap)</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>InventorySort</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>Ordina automaticamente gli oggetti nell'inventario e nei contenitori</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>Batch 2026-08 (Roadmap)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>Combat</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>BedTrap</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Piazza ed esplode automaticamente i letti nel Nether/End per PvP</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
         <is>
           <t>Batch 2026-08 (Roadmap)</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>AutoBrewer</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Gestisce automaticamente l'inserimento di ingredienti e fiamme negli alambicchi</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>Mappatura Qwen3.8-max</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>AutoSmelter</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Automatizza l'inserimento di prodotti e carburante nei forni</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>Mappatura Qwen3.8-max</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>StrongholdFinder</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Calcola le coordinate X, Z della fortezza triangolando 2 Occhi di Ender</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>Mappatura Qwen3.8-max</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>PacketLogger</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Registra i pacchetti di rete C2S e S2C inviati/ricevuti per debug</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
         <is>
           <t>Mappatura Qwen3.8-max</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="5" t="inlineStr">
         <is>
           <t>ServerFinder</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>Scansiona IP in background alla ricerca di server Minecraft attivi</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>Mappatura Qwen3.8-max</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>Render</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>Waypoints</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>Consente di impostare e visualizzare marcatori 3D con fasci di luce beacon</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
         <is>
           <t>Mappatura Qwen3.8-max</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>NoChatReports</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Disabilita le firme digitali sui messaggi inviati in chat per la privacy</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>Mappatura Qwen3.8-max</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>Combat</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>BowAimbot</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>Mantiene la mira automatica con l'arco calcolando parabola e anticipo</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>Mappatura Qwen3.8-max</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>Movement</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>AutoWalk</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>Mantiene la camminata in avanti automatica</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>Mappatura Qwen3.8-max</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>World</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>PluginScanner</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Scansiona /plugins e comandi del server per identificare PEX, LuckPerms, etc.</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t>Aggiunto da Qwen2.5</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>AntiDetect</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>Spoofa il brand del client in vanilla e rimuove i payload fabric:*</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>Integrato</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>SeedCracker</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>SeedCrackerModule</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Modulo wrapper per SeedCrackerX integrato: cracking semi, comandi /seedcracker</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Integrato da SeedCrackerX</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>PermissionViewer</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Mostra info profilo client in chat (solo client-side, nessun accesso al server)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Aggiunto in sessione audit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(movement): add Gesu water-walking module
Walk on water surfaces: neutralizes sinking velocity at the fluid surface, claims onGround, optional surface speed boost, dive-on-sneak, jump impulse to leave the surface. Settings: surfaceSpeed (1.0-2.0), diveOnSneak.
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" style="4" min="1" max="1"/>
@@ -2114,6 +2114,33 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Gesu</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Permette di camminare sulla superficie dell'acqua (con sneak = immergersi)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Aggiunto sessione 2026-08-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
feat(render): add SpectatorDetector module and update checklist to 67 modules
</commit_message>
<xml_diff>
--- a/Aetheris_Checklist_Test.xlsx
+++ b/Aetheris_Checklist_Test.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" style="4" min="1" max="1"/>
@@ -2141,6 +2141,33 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Render</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SpectatorDetector</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Rileva i giocatori in modalita spettatore dalla tab list e avvisa in chat su entrate/uscite (possibili staffer)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Aggiunto sessione 2026-08-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>